<commit_message>
feat: add TAG column to contact import template files
Both contatos_modelo.xlsx and contatos_modelo.csv now include a 'tag'
column with example values (CLIENTE, LEAD, VIP). The backend import
already supported this column — only the template files were missing it.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/contatos_modelo.xlsx
+++ b/frontend/public/contatos_modelo.xlsx
@@ -397,11 +397,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D6"/>
   <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -412,6 +413,9 @@
         <v>telefone</v>
       </c>
       <c r="C1" t="str">
+        <v>tag</v>
+      </c>
+      <c r="D1" t="str">
         <v>observacoes</v>
       </c>
     </row>
@@ -420,10 +424,13 @@
         <v>João Silva</v>
       </c>
       <c r="B2" t="str">
-        <v>11999999999</v>
+        <v>35999990001</v>
       </c>
       <c r="C2" t="str">
-        <v>Cliente VIP</v>
+        <v>CLIENTE</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Cliente desde 2024</v>
       </c>
     </row>
     <row r="3">
@@ -431,26 +438,60 @@
         <v>Maria Souza</v>
       </c>
       <c r="B3" t="str">
-        <v>21988888888</v>
+        <v>11988880002</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>LEAD</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Interessada no produto X</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Pedro Lima</v>
+        <v>Pedro Costa</v>
       </c>
       <c r="B4" t="str">
-        <v>31977777777</v>
+        <v>21977770003</v>
       </c>
       <c r="C4" t="str">
-        <v>Lead quente</v>
+        <v>VIP</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Cliente premium</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Ana Lima</v>
+      </c>
+      <c r="B5" t="str">
+        <v>31966660004</v>
+      </c>
+      <c r="C5" t="str">
+        <v>LEAD</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Carlos Mendes</v>
+      </c>
+      <c r="B6" t="str">
+        <v>51955550005</v>
+      </c>
+      <c r="C6" t="str">
+        <v>CLIENTE</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Comprou em janeiro</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add email column to contact import (backend + templates)
- contactController importCSV: reads email/e-mail/e_mail column,
  validates format, stores on contact; duplicate merge preserves email
- contatos_modelo.xlsx and .csv: add email column with example values

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/contatos_modelo.xlsx
+++ b/frontend/public/contatos_modelo.xlsx
@@ -397,12 +397,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="30.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -413,9 +414,12 @@
         <v>telefone</v>
       </c>
       <c r="C1" t="str">
+        <v>email</v>
+      </c>
+      <c r="D1" t="str">
         <v>tag</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>observacoes</v>
       </c>
     </row>
@@ -427,9 +431,12 @@
         <v>35999990001</v>
       </c>
       <c r="C2" t="str">
+        <v>joao@email.com</v>
+      </c>
+      <c r="D2" t="str">
         <v>CLIENTE</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>Cliente desde 2024</v>
       </c>
     </row>
@@ -441,9 +448,12 @@
         <v>11988880002</v>
       </c>
       <c r="C3" t="str">
+        <v>maria@email.com</v>
+      </c>
+      <c r="D3" t="str">
         <v>LEAD</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>Interessada no produto X</v>
       </c>
     </row>
@@ -455,9 +465,12 @@
         <v>21977770003</v>
       </c>
       <c r="C4" t="str">
+        <v>pedro@email.com</v>
+      </c>
+      <c r="D4" t="str">
         <v>VIP</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>Cliente premium</v>
       </c>
     </row>
@@ -469,9 +482,12 @@
         <v>31966660004</v>
       </c>
       <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
         <v>LEAD</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v/>
       </c>
     </row>
@@ -483,15 +499,18 @@
         <v>51955550005</v>
       </c>
       <c r="C6" t="str">
+        <v>carlos@email.com</v>
+      </c>
+      <c r="D6" t="str">
         <v>CLIENTE</v>
       </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <v>Comprou em janeiro</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>